<commit_message>
Fin de posicion de formulas en tabla qto
</commit_message>
<xml_diff>
--- a/CreateSheet/files/qtoC3.xlsx
+++ b/CreateSheet/files/qtoC3.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="53">
   <si>
     <t>Inputs</t>
   </si>
@@ -151,28 +151,25 @@
     <t>Notes</t>
   </si>
   <si>
-    <t>CAPEX</t>
-  </si>
-  <si>
-    <t>Hughes Equipment</t>
-  </si>
-  <si>
-    <t>VSAT</t>
-  </si>
-  <si>
-    <t>1505216-0332</t>
-  </si>
-  <si>
-    <t>HT2010</t>
-  </si>
-  <si>
-    <t>HT2010 Consumer Broadband Satellite Router, Ka Band only</t>
-  </si>
-  <si>
-    <t>Unit</t>
-  </si>
-  <si>
-    <t>NRC</t>
+    <t>1111</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>qqqqq+qqq</t>
+  </si>
+  <si>
+    <t>11</t>
+  </si>
+  <si>
+    <t>www</t>
+  </si>
+  <si>
+    <t>22</t>
+  </si>
+  <si>
+    <t>122</t>
   </si>
 </sst>
 </file>
@@ -301,8 +298,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" name="Qto" displayName="Qto" ref="A24:X29" totalsRowShown="1" headerRowCount="1">
-  <autoFilter ref="A24:X29">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" name="Qto" displayName="Qto" ref="A24:X26" totalsRowShown="1" headerRowCount="1">
+  <autoFilter ref="A24:X26">
     <filterColumn colId="0" hiddenButton="0"/>
     <filterColumn colId="1" hiddenButton="0"/>
     <filterColumn colId="2" hiddenButton="0"/>
@@ -680,7 +677,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:X29"/>
+  <dimension ref="A1:X26"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="2" max="2" width="27" customWidth="1"/>
@@ -925,7 +922,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="25" ht="13" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A25" s="7" t="s">
         <v>46</v>
       </c>
@@ -933,171 +930,146 @@
         <v>47</v>
       </c>
       <c r="C25" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="D25" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="D25" s="7" t="s">
+      <c r="E25" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="F25" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="E25" s="7" t="s">
+      <c r="G25" s="7">
+        <v>22</v>
+      </c>
+      <c r="H25" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="I25" s="7">
+        <v>11</v>
+      </c>
+      <c r="J25" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="F25" s="7" t="s">
+      <c r="K25" s="7">
+        <f>[[Unit Cost]]/0.7</f>
+      </c>
+      <c r="L25">
+        <f>[[Unit Price]]*(1-[Discount])</f>
+      </c>
+      <c r="M25">
+        <f>IF([Type]=1,$C$19,1)*[[Unit Disc. Price]]*[Qty]</f>
+      </c>
+      <c r="N25" s="7">
+        <v>54</v>
+      </c>
+      <c r="O25">
+        <f>IF([Type]="OPEX",$C$19,1)*[[Unit Cost]]*[Qty]
+</f>
+      </c>
+      <c r="P25">
+        <f>1-([[Ext. Cost]]/[[Ext. Disc. Price]])</f>
+      </c>
+      <c r="Q25" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="R25">
+        <f>[[Ext. Disc. Price]]/$C$7/$C$19</f>
+      </c>
+      <c r="S25">
+        <f>[[Ext. Cost]]/$C$7/$C$19</f>
+      </c>
+      <c r="T25">
+        <f>[[Ext. Disc. Price]]/$C$13/$C$19</f>
+      </c>
+      <c r="U25">
+        <f>[[Ext. Cost]]/$C$13/$C$19</f>
+      </c>
+      <c r="V25">
+        <f>IF(AND([Type]="CAPEX",[[Finance?]]="MRC"),PMT($C$21/12,$C$19,-[[Ext. Disc. Price]]),0)</f>
+      </c>
+      <c r="W25">
+        <f>IF(AND([Type]="CAPEX",[[Finance?]]="MRC"),PMT($C$21/12,$C$19,-[[Ext. Disc. Price]])/$C$7,IF([Type]="OPEX",[[Ext. Disc. Price]]/$C$7/$C$19,0))</f>
+      </c>
+      <c r="X25" s="7" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="26" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A26" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="G25" s="7">
-        <v>1204</v>
-      </c>
-      <c r="H25" s="7" t="s">
+      <c r="B26" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="C26" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="D26" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="E26" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="F26" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="G26" s="7">
+        <v>2</v>
+      </c>
+      <c r="H26" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="I26" s="7">
+        <v>11</v>
+      </c>
+      <c r="J26" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="I25" s="7">
-        <v>0</v>
-      </c>
-      <c r="J25" s="7" t="s">
-        <v>53</v>
-      </c>
-      <c r="K25" s="7">
-        <f>N25/0.7</f>
-      </c>
-    </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
-        <v>46</v>
-      </c>
-      <c r="B26" t="s">
-        <v>47</v>
-      </c>
-      <c r="C26" t="s">
-        <v>48</v>
-      </c>
-      <c r="D26" t="s">
-        <v>49</v>
-      </c>
-      <c r="E26" t="s">
-        <v>50</v>
-      </c>
-      <c r="F26" t="s">
-        <v>51</v>
-      </c>
-      <c r="G26">
-        <v>1204</v>
-      </c>
-      <c r="H26" t="s">
-        <v>52</v>
-      </c>
-      <c r="I26">
-        <v>0</v>
-      </c>
-      <c r="J26" t="s">
-        <v>53</v>
-      </c>
-      <c r="K26">
-        <v>85.08</v>
-      </c>
-    </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
-        <v>46</v>
-      </c>
-      <c r="B27" t="s">
-        <v>47</v>
-      </c>
-      <c r="C27" t="s">
-        <v>48</v>
-      </c>
-      <c r="D27" t="s">
-        <v>49</v>
-      </c>
-      <c r="E27" t="s">
-        <v>50</v>
-      </c>
-      <c r="F27" t="s">
-        <v>51</v>
-      </c>
-      <c r="G27">
-        <v>1204</v>
-      </c>
-      <c r="H27" t="s">
-        <v>52</v>
-      </c>
-      <c r="I27">
-        <v>0</v>
-      </c>
-      <c r="J27" t="s">
-        <v>53</v>
-      </c>
-      <c r="K27">
-        <v>85.08</v>
-      </c>
-    </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
-        <v>46</v>
-      </c>
-      <c r="B28" t="s">
-        <v>47</v>
-      </c>
-      <c r="C28" t="s">
-        <v>48</v>
-      </c>
-      <c r="D28" t="s">
-        <v>49</v>
-      </c>
-      <c r="E28" t="s">
-        <v>50</v>
-      </c>
-      <c r="F28" t="s">
-        <v>51</v>
-      </c>
-      <c r="G28">
-        <v>1204</v>
-      </c>
-      <c r="H28" t="s">
-        <v>52</v>
-      </c>
-      <c r="I28">
-        <v>0</v>
-      </c>
-      <c r="J28" t="s">
-        <v>53</v>
-      </c>
-      <c r="K28">
-        <v>85.08</v>
-      </c>
-    </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A29" t="s">
-        <v>46</v>
-      </c>
-      <c r="B29" t="s">
-        <v>47</v>
-      </c>
-      <c r="C29" t="s">
-        <v>48</v>
-      </c>
-      <c r="D29" t="s">
-        <v>49</v>
-      </c>
-      <c r="E29" t="s">
-        <v>50</v>
-      </c>
-      <c r="F29" t="s">
-        <v>51</v>
-      </c>
-      <c r="G29">
-        <v>1204</v>
-      </c>
-      <c r="H29" t="s">
-        <v>52</v>
-      </c>
-      <c r="I29">
-        <v>0</v>
-      </c>
-      <c r="J29" t="s">
-        <v>53</v>
-      </c>
-      <c r="K29">
-        <v>85.08</v>
+      <c r="K26" s="7">
+        <f>[[Unit Cost]]/0.7</f>
+      </c>
+      <c r="L26">
+        <f>[[Unit Price]]*(1-[Discount])</f>
+      </c>
+      <c r="M26">
+        <f>IF([Type]=1,$C$19,1)*[[Unit Disc. Price]]*[Qty]</f>
+      </c>
+      <c r="N26" s="7">
+        <v>54</v>
+      </c>
+      <c r="O26">
+        <f>IF([Type]="OPEX",$C$19,1)*[[Unit Cost]]*[Qty]
+</f>
+      </c>
+      <c r="P26">
+        <f>1-([[Ext. Cost]]/[[Ext. Disc. Price]])</f>
+      </c>
+      <c r="Q26" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="R26">
+        <f>[[Ext. Disc. Price]]/$C$7/$C$19</f>
+      </c>
+      <c r="S26">
+        <f>[[Ext. Cost]]/$C$7/$C$19</f>
+      </c>
+      <c r="T26">
+        <f>[[Ext. Disc. Price]]/$C$13/$C$19</f>
+      </c>
+      <c r="U26">
+        <f>[[Ext. Cost]]/$C$13/$C$19</f>
+      </c>
+      <c r="V26">
+        <f>IF(AND([Type]="CAPEX",[[Finance?]]="MRC"),PMT($C$21/12,$C$19,-[[Ext. Disc. Price]]),0)</f>
+      </c>
+      <c r="W26">
+        <f>IF(AND([Type]="CAPEX",[[Finance?]]="MRC"),PMT($C$21/12,$C$19,-[[Ext. Disc. Price]])/$C$7,IF([Type]="OPEX",[[Ext. Disc. Price]]/$C$7/$C$19,0))</f>
+      </c>
+      <c r="X26" s="7" t="s">
+        <v>47</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fin Tabla de Qto
</commit_message>
<xml_diff>
--- a/CreateSheet/files/qtoC3.xlsx
+++ b/CreateSheet/files/qtoC3.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="60">
   <si>
     <t>Inputs</t>
   </si>
@@ -19,18 +19,36 @@
     <t>Client:</t>
   </si>
   <si>
+    <t/>
+  </si>
+  <si>
     <t>Country:</t>
   </si>
   <si>
     <t>Proposal Manager:</t>
   </si>
   <si>
+    <t>PRICE</t>
+  </si>
+  <si>
+    <t>COST</t>
+  </si>
+  <si>
+    <t>MARGIN</t>
+  </si>
+  <si>
     <t>HUGHES T19 Number of Sites:</t>
   </si>
   <si>
+    <t>CAPEX</t>
+  </si>
+  <si>
     <t>Sites out of coverage:</t>
   </si>
   <si>
+    <t>OPEX</t>
+  </si>
+  <si>
     <t>Number of Sites:</t>
   </si>
   <si>
@@ -52,6 +70,12 @@
     <t>Total Ka band Capacity (Mbps):</t>
   </si>
   <si>
+    <t>Price x Site x Month</t>
+  </si>
+  <si>
+    <t>Cost x Site x Month</t>
+  </si>
+  <si>
     <t>Average Mbps per Site:</t>
   </si>
   <si>
@@ -152,9 +176,6 @@
   </si>
   <si>
     <t>1111</t>
-  </si>
-  <si>
-    <t/>
   </si>
   <si>
     <t>qqqqq+qqq</t>
@@ -176,7 +197,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="6" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* (#,##0.00);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
+  </numFmts>
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -202,6 +226,11 @@
     </font>
     <font>
       <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
       <sz val="10"/>
       <name val="Calibri"/>
     </font>
@@ -210,7 +239,7 @@
       <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -230,6 +259,16 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="D9D9D9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="B4C6E7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="F8CBAD"/>
       </patternFill>
     </fill>
   </fills>
@@ -259,7 +298,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="bottom"/>
@@ -271,13 +310,34 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="bottom"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="6" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="6" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="6" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -692,6 +752,13 @@
     <col min="13" max="13" width="16" customWidth="1"/>
     <col min="14" max="14" width="12" customWidth="1"/>
     <col min="15" max="15" width="13.5" customWidth="1"/>
+    <col min="16" max="16" width="14" customWidth="1"/>
+    <col min="17" max="17" width="10" customWidth="1"/>
+    <col min="18" max="19" width="22" customWidth="1"/>
+    <col min="20" max="21" width="24" customWidth="1"/>
+    <col min="22" max="22" width="17" customWidth="1"/>
+    <col min="23" max="23" width="28" customWidth="1"/>
+    <col min="24" max="24" width="10" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
@@ -706,370 +773,463 @@
         <v>1</v>
       </c>
       <c r="B2" s="3"/>
-      <c r="C2" s="4"/>
+      <c r="C2" s="4" t="s">
+        <v>2</v>
+      </c>
     </row>
     <row r="3" ht="12" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B3" s="3"/>
-      <c r="C3" s="4"/>
-    </row>
-    <row r="4" ht="15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C3" s="4" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" ht="15" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B4" s="3"/>
-      <c r="C4" s="4"/>
-    </row>
-    <row r="5" ht="15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C4" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5" ht="15" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="B5" s="3"/>
-      <c r="C5" s="4"/>
-    </row>
-    <row r="6" ht="15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C5" s="4">
+        <v>1</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F5">
+        <f>SUMIF(A24:A40,"CAPEX",M24:M40)</f>
+      </c>
+      <c r="G5">
+        <f>SUMIF(A24:A40,"CAPEX",O24:O40)</f>
+      </c>
+      <c r="H5">
+        <f>1-(G5/F5)</f>
+      </c>
+    </row>
+    <row r="6" ht="15" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="B6" s="3"/>
-      <c r="C6" s="4"/>
-    </row>
-    <row r="7" ht="15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C6" s="4">
+        <v>0</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="F6">
+        <f>SUMIF(A24:A40,"OPEX",M24:M40)</f>
+      </c>
+      <c r="G6">
+        <f>SUMIF(A24:A40,"OPEX",O24:O40)</f>
+      </c>
+      <c r="H6">
+        <f>1-(G6/F6)</f>
+      </c>
+    </row>
+    <row r="7" ht="15" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="B7" s="3"/>
-      <c r="C7" s="4"/>
+      <c r="C7" s="4">
+        <v>1111</v>
+      </c>
+      <c r="F7">
+        <f>SUM(F5:F6)</f>
+      </c>
+      <c r="G7">
+        <f>SUM(G5:G6)</f>
+      </c>
+      <c r="H7">
+        <f>1-(G7/F7)</f>
+      </c>
     </row>
     <row r="8" ht="12" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="B8" s="3"/>
-      <c r="C8" s="4"/>
+      <c r="C8" s="4">
+        <v>0</v>
+      </c>
     </row>
     <row r="9" ht="12" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="B9" s="3"/>
-      <c r="C9" s="4"/>
+      <c r="C9" s="4">
+        <v>0</v>
+      </c>
     </row>
     <row r="10" ht="12" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="B10" s="3"/>
-      <c r="C10" s="4"/>
+      <c r="C10" s="4" t="s">
+        <v>2</v>
+      </c>
     </row>
     <row r="11" ht="12" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="B11" s="3"/>
-      <c r="C11" s="4"/>
+      <c r="C11" s="4">
+        <v>0</v>
+      </c>
     </row>
     <row r="12" ht="12" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="B12" s="3"/>
-      <c r="C12" s="4"/>
-    </row>
-    <row r="13" ht="15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C12" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" ht="15" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="B13" s="3"/>
-      <c r="C13" s="4"/>
+      <c r="C13" s="4">
+        <v>11111</v>
+      </c>
+      <c r="F13" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="G13" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="H13" s="5" t="s">
+        <v>7</v>
+      </c>
     </row>
     <row r="14" ht="15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="B14" s="3"/>
-      <c r="C14" s="4"/>
+      <c r="C14" s="4">
+        <v>0</v>
+      </c>
     </row>
     <row r="15" ht="12" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="B15" s="3"/>
-      <c r="C15" s="4"/>
+      <c r="C15" s="4">
+        <v>0</v>
+      </c>
     </row>
     <row r="16" ht="12" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="B16" s="3"/>
-      <c r="C16" s="4"/>
+      <c r="C16" s="4">
+        <v>0</v>
+      </c>
     </row>
     <row r="17" ht="12" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="B17" s="3"/>
-      <c r="C17" s="4"/>
+      <c r="C17" s="4">
+        <v>0</v>
+      </c>
     </row>
     <row r="18" ht="12" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="B18" s="3"/>
-      <c r="C18" s="4"/>
+      <c r="C18" s="4">
+        <v>0</v>
+      </c>
     </row>
     <row r="19" ht="12" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="B19" s="3"/>
-      <c r="C19" s="4"/>
+      <c r="C19" s="4">
+        <v>11</v>
+      </c>
     </row>
     <row r="20" ht="12" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="B20" s="3"/>
-      <c r="C20" s="4"/>
+      <c r="C20" s="4">
+        <v>0</v>
+      </c>
     </row>
     <row r="21" ht="12" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="B21" s="3"/>
-      <c r="C21" s="4"/>
+      <c r="C21" s="4">
+        <v>12</v>
+      </c>
     </row>
     <row r="22" ht="12" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A22" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="B22" s="5"/>
-      <c r="C22" s="4"/>
+      <c r="A22" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B22" s="6"/>
+      <c r="C22" s="4">
+        <v>0</v>
+      </c>
     </row>
     <row r="24" ht="13" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A24" s="6" t="s">
+      <c r="A24" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="B24" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="C24" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="D24" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="E24" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="F24" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="G24" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="H24" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="I24" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="J24" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="K24" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="L24" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="M24" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="N24" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="O24" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="P24" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="Q24" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="R24" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="S24" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="T24" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="U24" s="8" t="s">
+        <v>50</v>
+      </c>
+      <c r="V24" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="W24" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="X24" s="7" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="25" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A25" s="9" t="s">
+        <v>54</v>
+      </c>
+      <c r="B25" s="9" t="s">
+        <v>2</v>
+      </c>
+      <c r="C25" s="9" t="s">
+        <v>2</v>
+      </c>
+      <c r="D25" s="9" t="s">
+        <v>55</v>
+      </c>
+      <c r="E25" s="9" t="s">
+        <v>2</v>
+      </c>
+      <c r="F25" s="9" t="s">
+        <v>56</v>
+      </c>
+      <c r="G25" s="10">
         <v>22</v>
       </c>
-      <c r="B24" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="C24" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="D24" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="E24" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="F24" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="G24" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="H24" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="I24" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="J24" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="K24" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="L24" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="M24" s="6" t="s">
-        <v>34</v>
-      </c>
-      <c r="N24" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="O24" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="P24" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="Q24" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="R24" s="6" t="s">
-        <v>39</v>
-      </c>
-      <c r="S24" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="T24" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="U24" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="V24" s="6" t="s">
-        <v>43</v>
-      </c>
-      <c r="W24" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="X24" s="6" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="25" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A25" s="7" t="s">
-        <v>46</v>
-      </c>
-      <c r="B25" s="7" t="s">
-        <v>47</v>
-      </c>
-      <c r="C25" s="7" t="s">
-        <v>47</v>
-      </c>
-      <c r="D25" s="7" t="s">
-        <v>48</v>
-      </c>
-      <c r="E25" s="7" t="s">
-        <v>47</v>
-      </c>
-      <c r="F25" s="7" t="s">
-        <v>49</v>
-      </c>
-      <c r="G25" s="7">
-        <v>22</v>
-      </c>
-      <c r="H25" s="7" t="s">
-        <v>47</v>
-      </c>
-      <c r="I25" s="7">
+      <c r="H25" s="9" t="s">
+        <v>2</v>
+      </c>
+      <c r="I25" s="11">
         <v>11</v>
       </c>
-      <c r="J25" s="7" t="s">
-        <v>50</v>
-      </c>
-      <c r="K25" s="7">
+      <c r="J25" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="K25" s="12">
         <f>[[Unit Cost]]/0.7</f>
       </c>
-      <c r="L25">
+      <c r="L25" s="13">
         <f>[[Unit Price]]*(1-[Discount])</f>
       </c>
-      <c r="M25">
+      <c r="M25" s="13">
         <f>IF([Type]=1,$C$19,1)*[[Unit Disc. Price]]*[Qty]</f>
       </c>
-      <c r="N25" s="7">
+      <c r="N25" s="12">
         <v>54</v>
       </c>
-      <c r="O25">
+      <c r="O25" s="13">
         <f>IF([Type]="OPEX",$C$19,1)*[[Unit Cost]]*[Qty]
 </f>
       </c>
-      <c r="P25">
+      <c r="P25" s="14">
         <f>1-([[Ext. Cost]]/[[Ext. Disc. Price]])</f>
       </c>
-      <c r="Q25" s="7" t="s">
-        <v>47</v>
-      </c>
-      <c r="R25">
+      <c r="Q25" s="9" t="s">
+        <v>2</v>
+      </c>
+      <c r="R25" s="13">
         <f>[[Ext. Disc. Price]]/$C$7/$C$19</f>
       </c>
-      <c r="S25">
+      <c r="S25" s="13">
         <f>[[Ext. Cost]]/$C$7/$C$19</f>
       </c>
-      <c r="T25">
+      <c r="T25" s="13">
         <f>[[Ext. Disc. Price]]/$C$13/$C$19</f>
       </c>
-      <c r="U25">
+      <c r="U25" s="13">
         <f>[[Ext. Cost]]/$C$13/$C$19</f>
       </c>
-      <c r="V25">
+      <c r="V25" s="13">
         <f>IF(AND([Type]="CAPEX",[[Finance?]]="MRC"),PMT($C$21/12,$C$19,-[[Ext. Disc. Price]]),0)</f>
       </c>
-      <c r="W25">
+      <c r="W25" s="13">
         <f>IF(AND([Type]="CAPEX",[[Finance?]]="MRC"),PMT($C$21/12,$C$19,-[[Ext. Disc. Price]])/$C$7,IF([Type]="OPEX",[[Ext. Disc. Price]]/$C$7/$C$19,0))</f>
       </c>
-      <c r="X25" s="7" t="s">
-        <v>47</v>
+      <c r="X25" s="9" t="s">
+        <v>2</v>
       </c>
     </row>
     <row r="26" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A26" s="7" t="s">
-        <v>51</v>
-      </c>
-      <c r="B26" s="7" t="s">
-        <v>47</v>
-      </c>
-      <c r="C26" s="7" t="s">
-        <v>47</v>
-      </c>
-      <c r="D26" s="7" t="s">
-        <v>49</v>
-      </c>
-      <c r="E26" s="7" t="s">
-        <v>47</v>
-      </c>
-      <c r="F26" s="7" t="s">
-        <v>47</v>
-      </c>
-      <c r="G26" s="7">
-        <v>2</v>
-      </c>
-      <c r="H26" s="7" t="s">
-        <v>47</v>
-      </c>
-      <c r="I26" s="7">
+      <c r="A26" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="B26" s="9" t="s">
+        <v>2</v>
+      </c>
+      <c r="C26" s="9" t="s">
+        <v>2</v>
+      </c>
+      <c r="D26" s="9" t="s">
+        <v>56</v>
+      </c>
+      <c r="E26" s="9" t="s">
+        <v>2</v>
+      </c>
+      <c r="F26" s="9" t="s">
+        <v>2</v>
+      </c>
+      <c r="G26" s="10">
+        <v>2</v>
+      </c>
+      <c r="H26" s="9" t="s">
+        <v>2</v>
+      </c>
+      <c r="I26" s="11">
         <v>11</v>
       </c>
-      <c r="J26" s="7" t="s">
-        <v>52</v>
-      </c>
-      <c r="K26" s="7">
+      <c r="J26" s="9" t="s">
+        <v>59</v>
+      </c>
+      <c r="K26" s="12">
         <f>[[Unit Cost]]/0.7</f>
       </c>
-      <c r="L26">
+      <c r="L26" s="13">
         <f>[[Unit Price]]*(1-[Discount])</f>
       </c>
-      <c r="M26">
+      <c r="M26" s="13">
         <f>IF([Type]=1,$C$19,1)*[[Unit Disc. Price]]*[Qty]</f>
       </c>
-      <c r="N26" s="7">
+      <c r="N26" s="12">
         <v>54</v>
       </c>
-      <c r="O26">
+      <c r="O26" s="13">
         <f>IF([Type]="OPEX",$C$19,1)*[[Unit Cost]]*[Qty]
 </f>
       </c>
-      <c r="P26">
+      <c r="P26" s="14">
         <f>1-([[Ext. Cost]]/[[Ext. Disc. Price]])</f>
       </c>
-      <c r="Q26" s="7" t="s">
-        <v>47</v>
-      </c>
-      <c r="R26">
+      <c r="Q26" s="9" t="s">
+        <v>2</v>
+      </c>
+      <c r="R26" s="13">
         <f>[[Ext. Disc. Price]]/$C$7/$C$19</f>
       </c>
-      <c r="S26">
+      <c r="S26" s="13">
         <f>[[Ext. Cost]]/$C$7/$C$19</f>
       </c>
-      <c r="T26">
+      <c r="T26" s="13">
         <f>[[Ext. Disc. Price]]/$C$13/$C$19</f>
       </c>
-      <c r="U26">
+      <c r="U26" s="13">
         <f>[[Ext. Cost]]/$C$13/$C$19</f>
       </c>
-      <c r="V26">
+      <c r="V26" s="13">
         <f>IF(AND([Type]="CAPEX",[[Finance?]]="MRC"),PMT($C$21/12,$C$19,-[[Ext. Disc. Price]]),0)</f>
       </c>
-      <c r="W26">
+      <c r="W26" s="13">
         <f>IF(AND([Type]="CAPEX",[[Finance?]]="MRC"),PMT($C$21/12,$C$19,-[[Ext. Disc. Price]])/$C$7,IF([Type]="OPEX",[[Ext. Disc. Price]]/$C$7/$C$19,0))</f>
       </c>
-      <c r="X26" s="7" t="s">
-        <v>47</v>
+      <c r="X26" s="9" t="s">
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>